<commit_message>
DC-3: Representante Legal + celdas amarillas + logo + instrucciones en negritas + leyenda
- DC-3: nuevo orden de columnas con Representante Legal (después de RFC)
- 6 primeros campos en amarillo (los llena el cliente del cliente)
- 8 siguientes en blanco (los llena AGASI)
- Logo AGASI como imagen flotante en esquina superior izquierda
- Instrucciones en formato lista con bullets
- Sección '¿QUIÉN LLENA CADA CAMPO?' con leyenda amarillo/blanco
- Instrucciones en negritas (no itálica)
- Mini-leyenda 💡 al inicio (misma celda mergeada): 'haz más grande la celda'
- Tabla arranca en columna A (logo no ocupa columna)
- Configuración de impresión: landscape, headers repetidos, márgenes normales
- build.spec: detección multi-plataforma de Playwright, greenlet en hiddenimports
- Workflow: genera icono placeholder si no existe
</commit_message>
<xml_diff>
--- a/static/ejemplo_certificados.xlsx
+++ b/static/ejemplo_certificados.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Participantes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Plantilla Reconocimiento" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Plantilla Reconocimiento'!$4:$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +27,50 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A4786"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A4786"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +78,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -122,6 +187,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="857250" cy="314325"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -413,262 +508,172 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plantilla Reconocimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>💡 Si no ves todo el texto, haz más grande la celda para ver todas las instrucciones completas.
+INSTRUCCIONES:
+• Complete los datos de los participantes.
+• El campo NOMBRE debe ir como: Apellido Paterno + Apellido Materno + Nombre(s)   Ej: López Hernández María Fernanda
+• La fila de ejemplo debe borrarse antes de procesar.
+• La columna FOLIO es opcional — si la deja vacía, el sistema asigna una automáticamente.
+─── ¿QUIÉN LLENA CADA CAMPO? ───
+Todos los campos los llena el CLIENTE (usted).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Nombre Completo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Curso</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Duracion (hrs)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Lugar</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Folio</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Lugar</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Empresa</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>María Fernanda López Hernández</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>López Hernández María Fernanda</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Seguridad Industrial y Protección Civil</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>40</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>15/06/2026</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>AG-001</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Ing. Roberto Martínez</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Pachuca, Hidalgo</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Industrias Peoles SAB de CV</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Carlos Alberto Mendoza Ruiz</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Manejo de Materiales Peligrosos</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>16/06/2026</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>AG-002</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Ing. Roberto Martínez</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Pachuca, Hidalgo</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Industrias Peoles SAB de CV</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Juan Pérez García</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Primeros Auxilios y RCP</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>16</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>17/06/2026</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>AG-003</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Dra. Ana Ruiz</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Pachuca, Hidalgo</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>CEMEX México SAB de CV</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ana Sofía Ramírez Cruz</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ISO 14001:2015 Sistemas de Gestión Ambiental</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>32</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>18/06/2026</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>AG-004</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Ing. Alejandro García</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Pachuca, Hidalgo</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>CEMEX México SAB de CV</t>
-        </is>
-      </c>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Roberto González Silva</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Evaluación de Riesgos y Peligros en el Trabajo</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>19/06/2026</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>AG-005</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Ing. Roberto Martínez</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Pachuca, Hidalgo</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Intermex Manufactura SA de CV</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G3"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>